<commit_message>
Fix hooks, scripts and tracker after fact-check; remove superseded sales page (live version is in propeloseo-site)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019hJSE1uEJk8ZbR3doNaKwz
</commit_message>
<xml_diff>
--- a/drafts/tiktok-hook-tracker.xlsx
+++ b/drafts/tiktok-hook-tracker.xlsx
@@ -162,16 +162,16 @@
     <t xml:space="preserve">The page that was switched off</t>
   </si>
   <si>
-    <t xml:space="preserve">One of this site's best pages had been switched off.</t>
+    <t xml:space="preserve">A page with 4,201 impressions had been switched off.</t>
   </si>
   <si>
     <t xml:space="preserve">Winner bar</t>
   </si>
   <si>
-    <t xml:space="preserve">Two pages</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Two pages. Same visibility.</t>
+    <t xml:space="preserve">Two groups of searches</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Two groups of searches. Same impressions.</t>
   </si>
   <si>
     <t xml:space="preserve">Best watch %</t>
@@ -189,7 +189,7 @@
     <t xml:space="preserve">764 keywords</t>
   </si>
   <si>
-    <t xml:space="preserve">764 keywords. 98 clicks in sixteen months.</t>
+    <t xml:space="preserve">764 generic keywords.</t>
   </si>
   <si>
     <t xml:space="preserve">The blank doc</t>
@@ -198,22 +198,22 @@
     <t xml:space="preserve">After a traffic drop, most of us open a blank doc and start rewriting.</t>
   </si>
   <si>
-    <t xml:space="preserve">Page one, no clicks</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Forty of this site's pages were already on page one of Google.</t>
+    <t xml:space="preserve">The legit pages</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The pages answering "is this site legit?" had 3 or 4 internal links.</t>
   </si>
   <si>
     <t xml:space="preserve">The bots</t>
   </si>
   <si>
-    <t xml:space="preserve">Part of this site's visibility loss wasn't people at all.</t>
+    <t xml:space="preserve">Part of this site's drop in impressions looked like bots, not people.</t>
   </si>
   <si>
     <t xml:space="preserve">Read the data</t>
   </si>
   <si>
-    <t xml:space="preserve">The usual advice is publish more.</t>
+    <t xml:space="preserve">The usual advice after a drop is publish more.</t>
   </si>
   <si>
     <t xml:space="preserve">How to use this tracker</t>
@@ -394,8 +394,12 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -403,7 +407,7 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -411,35 +415,35 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="167" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="168" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="169" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -698,574 +702,574 @@
   <dimension ref="A1:W11"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="4"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="60"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="17"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="10" style="0" width="9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="0" width="9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="22" min="22" style="0" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="23" min="23" style="0" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="60"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="17"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="10" style="1" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="1" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="1" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="1" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="22" min="22" style="1" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="23" min="23" style="1" width="24"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+    <row r="1" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" s="2" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="n">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="D2" s="2" t="n">
-        <v>42</v>
-      </c>
-      <c r="E2" s="4" t="n">
+      <c r="D2" s="3" t="n">
+        <v>35</v>
+      </c>
+      <c r="E2" s="5" t="n">
         <f aca="false">D2*0.315</f>
-        <v>13.23</v>
-      </c>
-      <c r="F2" s="5"/>
-      <c r="G2" s="6"/>
-      <c r="H2" s="6"/>
-      <c r="I2" s="6"/>
-      <c r="J2" s="7" t="str">
+        <v>11.025</v>
+      </c>
+      <c r="F2" s="6"/>
+      <c r="G2" s="7"/>
+      <c r="H2" s="7"/>
+      <c r="I2" s="7"/>
+      <c r="J2" s="8" t="str">
         <f aca="false">IF(OR(H2="",I2=""),"",I2/E2)</f>
         <v/>
       </c>
-      <c r="K2" s="6"/>
-      <c r="L2" s="6"/>
-      <c r="M2" s="6"/>
-      <c r="N2" s="6"/>
-      <c r="O2" s="6"/>
-      <c r="P2" s="6"/>
-      <c r="Q2" s="7" t="str">
+      <c r="K2" s="7"/>
+      <c r="L2" s="7"/>
+      <c r="M2" s="7"/>
+      <c r="N2" s="7"/>
+      <c r="O2" s="7"/>
+      <c r="P2" s="7"/>
+      <c r="Q2" s="8" t="str">
         <f aca="false">IF(OR(L2="",P2="",L2=0),"",P2/L2)</f>
         <v/>
       </c>
-      <c r="R2" s="8" t="str">
+      <c r="R2" s="9" t="str">
         <f aca="false">IF(OR(H2="",NOT(ISNUMBER($W$3)),$W$3=0),"",H2/$W$3)</f>
         <v/>
       </c>
-      <c r="S2" s="2" t="str">
+      <c r="S2" s="3" t="str">
         <f aca="false">IF(H2="","Not posted",IF(NOT(ISNUMBER($W$3)),"Insufficient evidence",IF(AND(H2&gt;=200,R2&gt;=1.5),"Provisional winner","Below bar")))</f>
         <v>Not posted</v>
       </c>
-      <c r="T2" s="6"/>
-      <c r="V2" s="9" t="s">
+      <c r="T2" s="7"/>
+      <c r="V2" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="W2" s="2" t="n">
+      <c r="W2" s="3" t="n">
         <f aca="false">COUNT(H2:H11)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="n">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="D3" s="2" t="n">
-        <v>36</v>
-      </c>
-      <c r="E3" s="4" t="n">
+      <c r="D3" s="3" t="n">
+        <v>38</v>
+      </c>
+      <c r="E3" s="5" t="n">
         <f aca="false">D3*0.315</f>
-        <v>11.34</v>
-      </c>
-      <c r="F3" s="5"/>
-      <c r="G3" s="6"/>
-      <c r="H3" s="6"/>
-      <c r="I3" s="6"/>
-      <c r="J3" s="7" t="str">
+        <v>11.97</v>
+      </c>
+      <c r="F3" s="6"/>
+      <c r="G3" s="7"/>
+      <c r="H3" s="7"/>
+      <c r="I3" s="7"/>
+      <c r="J3" s="8" t="str">
         <f aca="false">IF(OR(H3="",I3=""),"",I3/E3)</f>
         <v/>
       </c>
-      <c r="K3" s="6"/>
-      <c r="L3" s="6"/>
-      <c r="M3" s="6"/>
-      <c r="N3" s="6"/>
-      <c r="O3" s="6"/>
-      <c r="P3" s="6"/>
-      <c r="Q3" s="7" t="str">
+      <c r="K3" s="7"/>
+      <c r="L3" s="7"/>
+      <c r="M3" s="7"/>
+      <c r="N3" s="7"/>
+      <c r="O3" s="7"/>
+      <c r="P3" s="7"/>
+      <c r="Q3" s="8" t="str">
         <f aca="false">IF(OR(L3="",P3="",L3=0),"",P3/L3)</f>
         <v/>
       </c>
-      <c r="R3" s="8" t="str">
+      <c r="R3" s="9" t="str">
         <f aca="false">IF(OR(H3="",NOT(ISNUMBER($W$3)),$W$3=0),"",H3/$W$3)</f>
         <v/>
       </c>
-      <c r="S3" s="2" t="str">
+      <c r="S3" s="3" t="str">
         <f aca="false">IF(H3="","Not posted",IF(NOT(ISNUMBER($W$3)),"Insufficient evidence",IF(AND(H3&gt;=200,R3&gt;=1.5),"Provisional winner","Below bar")))</f>
         <v>Not posted</v>
       </c>
-      <c r="T3" s="6"/>
-      <c r="V3" s="9" t="s">
+      <c r="T3" s="7"/>
+      <c r="V3" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="W3" s="2" t="str">
+      <c r="W3" s="3" t="str">
         <f aca="false">IF(W2&gt;=5,MEDIAN(H2:H11),"Insufficient evidence (&lt;5)")</f>
         <v>Insufficient evidence (&lt;5)</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2" t="n">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="D4" s="2" t="n">
+      <c r="D4" s="3" t="n">
         <v>42</v>
       </c>
-      <c r="E4" s="4" t="n">
+      <c r="E4" s="5" t="n">
         <f aca="false">D4*0.315</f>
         <v>13.23</v>
       </c>
-      <c r="F4" s="5"/>
-      <c r="G4" s="6"/>
-      <c r="H4" s="6"/>
-      <c r="I4" s="6"/>
-      <c r="J4" s="7" t="str">
+      <c r="F4" s="6"/>
+      <c r="G4" s="7"/>
+      <c r="H4" s="7"/>
+      <c r="I4" s="7"/>
+      <c r="J4" s="8" t="str">
         <f aca="false">IF(OR(H4="",I4=""),"",I4/E4)</f>
         <v/>
       </c>
-      <c r="K4" s="6"/>
-      <c r="L4" s="6"/>
-      <c r="M4" s="6"/>
-      <c r="N4" s="6"/>
-      <c r="O4" s="6"/>
-      <c r="P4" s="6"/>
-      <c r="Q4" s="7" t="str">
+      <c r="K4" s="7"/>
+      <c r="L4" s="7"/>
+      <c r="M4" s="7"/>
+      <c r="N4" s="7"/>
+      <c r="O4" s="7"/>
+      <c r="P4" s="7"/>
+      <c r="Q4" s="8" t="str">
         <f aca="false">IF(OR(L4="",P4="",L4=0),"",P4/L4)</f>
         <v/>
       </c>
-      <c r="R4" s="8" t="str">
+      <c r="R4" s="9" t="str">
         <f aca="false">IF(OR(H4="",NOT(ISNUMBER($W$3)),$W$3=0),"",H4/$W$3)</f>
         <v/>
       </c>
-      <c r="S4" s="2" t="str">
+      <c r="S4" s="3" t="str">
         <f aca="false">IF(H4="","Not posted",IF(NOT(ISNUMBER($W$3)),"Insufficient evidence",IF(AND(H4&gt;=200,R4&gt;=1.5),"Provisional winner","Below bar")))</f>
         <v>Not posted</v>
       </c>
-      <c r="T4" s="6"/>
-      <c r="V4" s="9" t="s">
+      <c r="T4" s="7"/>
+      <c r="V4" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="W4" s="10" t="str">
+      <c r="W4" s="11" t="str">
         <f aca="false">IF(ISNUMBER(W3),MAX(200,1.5*W3),"")</f>
         <v/>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="2" t="n">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="D5" s="2" t="n">
-        <v>40</v>
-      </c>
-      <c r="E5" s="4" t="n">
+      <c r="D5" s="3" t="n">
+        <v>37</v>
+      </c>
+      <c r="E5" s="5" t="n">
         <f aca="false">D5*0.315</f>
-        <v>12.6</v>
-      </c>
-      <c r="F5" s="5"/>
-      <c r="G5" s="6"/>
-      <c r="H5" s="6"/>
-      <c r="I5" s="6"/>
-      <c r="J5" s="7" t="str">
+        <v>11.655</v>
+      </c>
+      <c r="F5" s="6"/>
+      <c r="G5" s="7"/>
+      <c r="H5" s="7"/>
+      <c r="I5" s="7"/>
+      <c r="J5" s="8" t="str">
         <f aca="false">IF(OR(H5="",I5=""),"",I5/E5)</f>
         <v/>
       </c>
-      <c r="K5" s="6"/>
-      <c r="L5" s="6"/>
-      <c r="M5" s="6"/>
-      <c r="N5" s="6"/>
-      <c r="O5" s="6"/>
-      <c r="P5" s="6"/>
-      <c r="Q5" s="7" t="str">
+      <c r="K5" s="7"/>
+      <c r="L5" s="7"/>
+      <c r="M5" s="7"/>
+      <c r="N5" s="7"/>
+      <c r="O5" s="7"/>
+      <c r="P5" s="7"/>
+      <c r="Q5" s="8" t="str">
         <f aca="false">IF(OR(L5="",P5="",L5=0),"",P5/L5)</f>
         <v/>
       </c>
-      <c r="R5" s="8" t="str">
+      <c r="R5" s="9" t="str">
         <f aca="false">IF(OR(H5="",NOT(ISNUMBER($W$3)),$W$3=0),"",H5/$W$3)</f>
         <v/>
       </c>
-      <c r="S5" s="2" t="str">
+      <c r="S5" s="3" t="str">
         <f aca="false">IF(H5="","Not posted",IF(NOT(ISNUMBER($W$3)),"Insufficient evidence",IF(AND(H5&gt;=200,R5&gt;=1.5),"Provisional winner","Below bar")))</f>
         <v>Not posted</v>
       </c>
-      <c r="T5" s="6"/>
-      <c r="V5" s="9" t="s">
+      <c r="T5" s="7"/>
+      <c r="V5" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="W5" s="7" t="str">
+      <c r="W5" s="8" t="str">
         <f aca="false">IF(COUNT(J2:J11)=0,"",MAX(J2:J11))</f>
         <v/>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="2" t="n">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="C6" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="D6" s="2" t="n">
-        <v>41</v>
-      </c>
-      <c r="E6" s="4" t="n">
+      <c r="D6" s="3" t="n">
+        <v>36</v>
+      </c>
+      <c r="E6" s="5" t="n">
         <f aca="false">D6*0.315</f>
-        <v>12.915</v>
-      </c>
-      <c r="F6" s="5"/>
-      <c r="G6" s="6"/>
-      <c r="H6" s="6"/>
-      <c r="I6" s="6"/>
-      <c r="J6" s="7" t="str">
+        <v>11.34</v>
+      </c>
+      <c r="F6" s="6"/>
+      <c r="G6" s="7"/>
+      <c r="H6" s="7"/>
+      <c r="I6" s="7"/>
+      <c r="J6" s="8" t="str">
         <f aca="false">IF(OR(H6="",I6=""),"",I6/E6)</f>
         <v/>
       </c>
-      <c r="K6" s="6"/>
-      <c r="L6" s="6"/>
-      <c r="M6" s="6"/>
-      <c r="N6" s="6"/>
-      <c r="O6" s="6"/>
-      <c r="P6" s="6"/>
-      <c r="Q6" s="7" t="str">
+      <c r="K6" s="7"/>
+      <c r="L6" s="7"/>
+      <c r="M6" s="7"/>
+      <c r="N6" s="7"/>
+      <c r="O6" s="7"/>
+      <c r="P6" s="7"/>
+      <c r="Q6" s="8" t="str">
         <f aca="false">IF(OR(L6="",P6="",L6=0),"",P6/L6)</f>
         <v/>
       </c>
-      <c r="R6" s="8" t="str">
+      <c r="R6" s="9" t="str">
         <f aca="false">IF(OR(H6="",NOT(ISNUMBER($W$3)),$W$3=0),"",H6/$W$3)</f>
         <v/>
       </c>
-      <c r="S6" s="2" t="str">
+      <c r="S6" s="3" t="str">
         <f aca="false">IF(H6="","Not posted",IF(NOT(ISNUMBER($W$3)),"Insufficient evidence",IF(AND(H6&gt;=200,R6&gt;=1.5),"Provisional winner","Below bar")))</f>
         <v>Not posted</v>
       </c>
-      <c r="T6" s="6"/>
-      <c r="V6" s="9" t="s">
+      <c r="T6" s="7"/>
+      <c r="V6" s="10" t="s">
         <v>34</v>
       </c>
-      <c r="W6" s="2" t="str">
+      <c r="W6" s="3" t="str">
         <f aca="false">IF(W5="","",INDEX(B2:B11,MATCH(W5,J2:J11,0)))</f>
         <v/>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="2" t="n">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="C7" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="D7" s="2" t="n">
-        <v>42</v>
-      </c>
-      <c r="E7" s="4" t="n">
+      <c r="D7" s="3" t="n">
+        <v>35</v>
+      </c>
+      <c r="E7" s="5" t="n">
         <f aca="false">D7*0.315</f>
-        <v>13.23</v>
-      </c>
-      <c r="F7" s="5"/>
-      <c r="G7" s="6"/>
-      <c r="H7" s="6"/>
-      <c r="I7" s="6"/>
-      <c r="J7" s="7" t="str">
+        <v>11.025</v>
+      </c>
+      <c r="F7" s="6"/>
+      <c r="G7" s="7"/>
+      <c r="H7" s="7"/>
+      <c r="I7" s="7"/>
+      <c r="J7" s="8" t="str">
         <f aca="false">IF(OR(H7="",I7=""),"",I7/E7)</f>
         <v/>
       </c>
-      <c r="K7" s="6"/>
-      <c r="L7" s="6"/>
-      <c r="M7" s="6"/>
-      <c r="N7" s="6"/>
-      <c r="O7" s="6"/>
-      <c r="P7" s="6"/>
-      <c r="Q7" s="7" t="str">
+      <c r="K7" s="7"/>
+      <c r="L7" s="7"/>
+      <c r="M7" s="7"/>
+      <c r="N7" s="7"/>
+      <c r="O7" s="7"/>
+      <c r="P7" s="7"/>
+      <c r="Q7" s="8" t="str">
         <f aca="false">IF(OR(L7="",P7="",L7=0),"",P7/L7)</f>
         <v/>
       </c>
-      <c r="R7" s="8" t="str">
+      <c r="R7" s="9" t="str">
         <f aca="false">IF(OR(H7="",NOT(ISNUMBER($W$3)),$W$3=0),"",H7/$W$3)</f>
         <v/>
       </c>
-      <c r="S7" s="2" t="str">
+      <c r="S7" s="3" t="str">
         <f aca="false">IF(H7="","Not posted",IF(NOT(ISNUMBER($W$3)),"Insufficient evidence",IF(AND(H7&gt;=200,R7&gt;=1.5),"Provisional winner","Below bar")))</f>
         <v>Not posted</v>
       </c>
-      <c r="T7" s="6"/>
-    </row>
-    <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="2" t="n">
+      <c r="T7" s="7"/>
+    </row>
+    <row r="8" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B8" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="C8" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="D8" s="2" t="n">
-        <v>41</v>
-      </c>
-      <c r="E8" s="4" t="n">
+      <c r="D8" s="3" t="n">
+        <v>42</v>
+      </c>
+      <c r="E8" s="5" t="n">
         <f aca="false">D8*0.315</f>
-        <v>12.915</v>
-      </c>
-      <c r="F8" s="5"/>
-      <c r="G8" s="6"/>
-      <c r="H8" s="6"/>
-      <c r="I8" s="6"/>
-      <c r="J8" s="7" t="str">
+        <v>13.23</v>
+      </c>
+      <c r="F8" s="6"/>
+      <c r="G8" s="7"/>
+      <c r="H8" s="7"/>
+      <c r="I8" s="7"/>
+      <c r="J8" s="8" t="str">
         <f aca="false">IF(OR(H8="",I8=""),"",I8/E8)</f>
         <v/>
       </c>
-      <c r="K8" s="6"/>
-      <c r="L8" s="6"/>
-      <c r="M8" s="6"/>
-      <c r="N8" s="6"/>
-      <c r="O8" s="6"/>
-      <c r="P8" s="6"/>
-      <c r="Q8" s="7" t="str">
+      <c r="K8" s="7"/>
+      <c r="L8" s="7"/>
+      <c r="M8" s="7"/>
+      <c r="N8" s="7"/>
+      <c r="O8" s="7"/>
+      <c r="P8" s="7"/>
+      <c r="Q8" s="8" t="str">
         <f aca="false">IF(OR(L8="",P8="",L8=0),"",P8/L8)</f>
         <v/>
       </c>
-      <c r="R8" s="8" t="str">
+      <c r="R8" s="9" t="str">
         <f aca="false">IF(OR(H8="",NOT(ISNUMBER($W$3)),$W$3=0),"",H8/$W$3)</f>
         <v/>
       </c>
-      <c r="S8" s="2" t="str">
+      <c r="S8" s="3" t="str">
         <f aca="false">IF(H8="","Not posted",IF(NOT(ISNUMBER($W$3)),"Insufficient evidence",IF(AND(H8&gt;=200,R8&gt;=1.5),"Provisional winner","Below bar")))</f>
         <v>Not posted</v>
       </c>
-      <c r="T8" s="6"/>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="2" t="n">
+      <c r="T8" s="7"/>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B9" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="C9" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="D9" s="2" t="n">
-        <v>39</v>
-      </c>
-      <c r="E9" s="4" t="n">
+      <c r="D9" s="3" t="n">
+        <v>35</v>
+      </c>
+      <c r="E9" s="5" t="n">
         <f aca="false">D9*0.315</f>
-        <v>12.285</v>
-      </c>
-      <c r="F9" s="5"/>
-      <c r="G9" s="6"/>
-      <c r="H9" s="6"/>
-      <c r="I9" s="6"/>
-      <c r="J9" s="7" t="str">
+        <v>11.025</v>
+      </c>
+      <c r="F9" s="6"/>
+      <c r="G9" s="7"/>
+      <c r="H9" s="7"/>
+      <c r="I9" s="7"/>
+      <c r="J9" s="8" t="str">
         <f aca="false">IF(OR(H9="",I9=""),"",I9/E9)</f>
         <v/>
       </c>
-      <c r="K9" s="6"/>
-      <c r="L9" s="6"/>
-      <c r="M9" s="6"/>
-      <c r="N9" s="6"/>
-      <c r="O9" s="6"/>
-      <c r="P9" s="6"/>
-      <c r="Q9" s="7" t="str">
+      <c r="K9" s="7"/>
+      <c r="L9" s="7"/>
+      <c r="M9" s="7"/>
+      <c r="N9" s="7"/>
+      <c r="O9" s="7"/>
+      <c r="P9" s="7"/>
+      <c r="Q9" s="8" t="str">
         <f aca="false">IF(OR(L9="",P9="",L9=0),"",P9/L9)</f>
         <v/>
       </c>
-      <c r="R9" s="8" t="str">
+      <c r="R9" s="9" t="str">
         <f aca="false">IF(OR(H9="",NOT(ISNUMBER($W$3)),$W$3=0),"",H9/$W$3)</f>
         <v/>
       </c>
-      <c r="S9" s="2" t="str">
+      <c r="S9" s="3" t="str">
         <f aca="false">IF(H9="","Not posted",IF(NOT(ISNUMBER($W$3)),"Insufficient evidence",IF(AND(H9&gt;=200,R9&gt;=1.5),"Provisional winner","Below bar")))</f>
         <v>Not posted</v>
       </c>
-      <c r="T9" s="6"/>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="2" t="n">
+      <c r="T9" s="7"/>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="3" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B10" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="C10" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="D10" s="2" t="n">
-        <v>37</v>
-      </c>
-      <c r="E10" s="4" t="n">
+      <c r="D10" s="3" t="n">
+        <v>42</v>
+      </c>
+      <c r="E10" s="5" t="n">
         <f aca="false">D10*0.315</f>
-        <v>11.655</v>
-      </c>
-      <c r="F10" s="5"/>
-      <c r="G10" s="6"/>
-      <c r="H10" s="6"/>
-      <c r="I10" s="6"/>
-      <c r="J10" s="7" t="str">
+        <v>13.23</v>
+      </c>
+      <c r="F10" s="6"/>
+      <c r="G10" s="7"/>
+      <c r="H10" s="7"/>
+      <c r="I10" s="7"/>
+      <c r="J10" s="8" t="str">
         <f aca="false">IF(OR(H10="",I10=""),"",I10/E10)</f>
         <v/>
       </c>
-      <c r="K10" s="6"/>
-      <c r="L10" s="6"/>
-      <c r="M10" s="6"/>
-      <c r="N10" s="6"/>
-      <c r="O10" s="6"/>
-      <c r="P10" s="6"/>
-      <c r="Q10" s="7" t="str">
+      <c r="K10" s="7"/>
+      <c r="L10" s="7"/>
+      <c r="M10" s="7"/>
+      <c r="N10" s="7"/>
+      <c r="O10" s="7"/>
+      <c r="P10" s="7"/>
+      <c r="Q10" s="8" t="str">
         <f aca="false">IF(OR(L10="",P10="",L10=0),"",P10/L10)</f>
         <v/>
       </c>
-      <c r="R10" s="8" t="str">
+      <c r="R10" s="9" t="str">
         <f aca="false">IF(OR(H10="",NOT(ISNUMBER($W$3)),$W$3=0),"",H10/$W$3)</f>
         <v/>
       </c>
-      <c r="S10" s="2" t="str">
+      <c r="S10" s="3" t="str">
         <f aca="false">IF(H10="","Not posted",IF(NOT(ISNUMBER($W$3)),"Insufficient evidence",IF(AND(H10&gt;=200,R10&gt;=1.5),"Provisional winner","Below bar")))</f>
         <v>Not posted</v>
       </c>
-      <c r="T10" s="6"/>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="2" t="n">
+      <c r="T10" s="7"/>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="3" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B11" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="C11" s="3" t="s">
+      <c r="C11" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="D11" s="2" t="n">
+      <c r="D11" s="3" t="n">
         <v>42</v>
       </c>
-      <c r="E11" s="4" t="n">
+      <c r="E11" s="5" t="n">
         <f aca="false">D11*0.315</f>
         <v>13.23</v>
       </c>
-      <c r="F11" s="5"/>
-      <c r="G11" s="6"/>
-      <c r="H11" s="6"/>
-      <c r="I11" s="6"/>
-      <c r="J11" s="7" t="str">
+      <c r="F11" s="6"/>
+      <c r="G11" s="7"/>
+      <c r="H11" s="7"/>
+      <c r="I11" s="7"/>
+      <c r="J11" s="8" t="str">
         <f aca="false">IF(OR(H11="",I11=""),"",I11/E11)</f>
         <v/>
       </c>
-      <c r="K11" s="6"/>
-      <c r="L11" s="6"/>
-      <c r="M11" s="6"/>
-      <c r="N11" s="6"/>
-      <c r="O11" s="6"/>
-      <c r="P11" s="6"/>
-      <c r="Q11" s="7" t="str">
+      <c r="K11" s="7"/>
+      <c r="L11" s="7"/>
+      <c r="M11" s="7"/>
+      <c r="N11" s="7"/>
+      <c r="O11" s="7"/>
+      <c r="P11" s="7"/>
+      <c r="Q11" s="8" t="str">
         <f aca="false">IF(OR(L11="",P11="",L11=0),"",P11/L11)</f>
         <v/>
       </c>
-      <c r="R11" s="8" t="str">
+      <c r="R11" s="9" t="str">
         <f aca="false">IF(OR(H11="",NOT(ISNUMBER($W$3)),$W$3=0),"",H11/$W$3)</f>
         <v/>
       </c>
-      <c r="S11" s="2" t="str">
+      <c r="S11" s="3" t="str">
         <f aca="false">IF(H11="","Not posted",IF(NOT(ISNUMBER($W$3)),"Insufficient evidence",IF(AND(H11&gt;=200,R11&gt;=1.5),"Provisional winner","Below bar")))</f>
         <v>Not posted</v>
       </c>
-      <c r="T11" s="6"/>
+      <c r="T11" s="7"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -1287,117 +1291,117 @@
   <dimension ref="A1:G16"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="95"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="2" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="95"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="2" style="1" width="16"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="9" t="s">
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="10" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2"/>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="s">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3"/>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="3" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2" t="s">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="3" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="2" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="3" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="2"/>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="9" t="s">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="3"/>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="10" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="2" t="s">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="3" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="2" t="s">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="3" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="2" t="s">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="3" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="2" t="s">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="3" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="2" t="s">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="3" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="2"/>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="9" t="s">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="3"/>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="10" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="9" t="s">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="B15" s="9" t="s">
+      <c r="B15" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="C15" s="9" t="s">
+      <c r="C15" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="D15" s="9" t="s">
+      <c r="D15" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="E15" s="9" t="s">
+      <c r="E15" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="F15" s="9" t="s">
+      <c r="F15" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="G15" s="9" t="s">
+      <c r="G15" s="10" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="11" t="s">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="12" t="s">
         <v>59</v>
       </c>
-      <c r="B16" s="11" t="s">
+      <c r="B16" s="12" t="s">
         <v>60</v>
       </c>
-      <c r="C16" s="11" t="n">
+      <c r="C16" s="12" t="n">
         <v>143</v>
       </c>
-      <c r="D16" s="11" t="n">
+      <c r="D16" s="12" t="n">
         <v>7.2</v>
       </c>
-      <c r="E16" s="11" t="n">
+      <c r="E16" s="12" t="n">
         <v>310</v>
       </c>
-      <c r="F16" s="11" t="n">
+      <c r="F16" s="12" t="n">
         <v>402</v>
       </c>
-      <c r="G16" s="11" t="n">
+      <c r="G16" s="12" t="n">
         <v>6</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Round client figures in hooks, scripts and tracker
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019hJSE1uEJk8ZbR3doNaKwz
</commit_message>
<xml_diff>
--- a/drafts/tiktok-hook-tracker.xlsx
+++ b/drafts/tiktok-hook-tracker.xlsx
@@ -162,7 +162,7 @@
     <t xml:space="preserve">The page that was switched off</t>
   </si>
   <si>
-    <t xml:space="preserve">A page with 4,201 impressions had been switched off.</t>
+    <t xml:space="preserve">A page with over 4,000 impressions had been switched off.</t>
   </si>
   <si>
     <t xml:space="preserve">Winner bar</t>
@@ -186,10 +186,10 @@
     <t xml:space="preserve">Hook with best watch %</t>
   </si>
   <si>
-    <t xml:space="preserve">764 keywords</t>
-  </si>
-  <si>
-    <t xml:space="preserve">764 generic keywords.</t>
+    <t xml:space="preserve">700 keywords</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Over 700 generic keywords.</t>
   </si>
   <si>
     <t xml:space="preserve">The blank doc</t>
@@ -201,7 +201,7 @@
     <t xml:space="preserve">The legit pages</t>
   </si>
   <si>
-    <t xml:space="preserve">The pages answering "is this site legit?" had 3 or 4 internal links.</t>
+    <t xml:space="preserve">The pages answering "is this site legit?" had fewer than 5 internal links.</t>
   </si>
   <si>
     <t xml:space="preserve">The bots</t>
@@ -797,11 +797,11 @@
         <v>21</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E2" s="5" t="n">
         <f aca="false">D2*0.315</f>
-        <v>11.025</v>
+        <v>11.34</v>
       </c>
       <c r="F2" s="6"/>
       <c r="G2" s="7"/>
@@ -901,11 +901,11 @@
         <v>27</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="E4" s="5" t="n">
         <f aca="false">D4*0.315</f>
-        <v>13.23</v>
+        <v>12.6</v>
       </c>
       <c r="F4" s="6"/>
       <c r="G4" s="7"/>
@@ -953,11 +953,11 @@
         <v>30</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="E5" s="5" t="n">
         <f aca="false">D5*0.315</f>
-        <v>11.655</v>
+        <v>12.285</v>
       </c>
       <c r="F5" s="6"/>
       <c r="G5" s="7"/>
@@ -1057,11 +1057,11 @@
         <v>36</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="E7" s="5" t="n">
         <f aca="false">D7*0.315</f>
-        <v>11.025</v>
+        <v>12.285</v>
       </c>
       <c r="F7" s="6"/>
       <c r="G7" s="7"/>
@@ -1192,11 +1192,11 @@
         <v>42</v>
       </c>
       <c r="D10" s="3" t="n">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="E10" s="5" t="n">
         <f aca="false">D10*0.315</f>
-        <v>13.23</v>
+        <v>10.08</v>
       </c>
       <c r="F10" s="6"/>
       <c r="G10" s="7"/>
@@ -1237,11 +1237,11 @@
         <v>44</v>
       </c>
       <c r="D11" s="3" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E11" s="5" t="n">
         <f aca="false">D11*0.315</f>
-        <v>13.23</v>
+        <v>12.915</v>
       </c>
       <c r="F11" s="6"/>
       <c r="G11" s="7"/>

</xml_diff>